<commit_message>
feat: conclui melhorias e calculos do AgenteCompara
</commit_message>
<xml_diff>
--- a/app/protected_files/templates/template_agente_compara.xlsx
+++ b/app/protected_files/templates/template_agente_compara.xlsx
@@ -17,13 +17,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,180 +418,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>transportadora</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_documento</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cidade_origem</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>uf_origem</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>cidade_destino</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>uf_destino</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>valor_nf</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>valor_frete</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>peso</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>modal</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>data_emissao</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>data_entrega</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Transportadora Exemplo A</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>NF-1001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Sao Paulo</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>RJ</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>12000.5</v>
-      </c>
-      <c r="H2" t="n">
-        <v>980.75</v>
-      </c>
-      <c r="I2" t="n">
-        <v>450</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>rodoviario</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>2026-01-10</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-01-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Transportadora Exemplo B</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CTE-2002</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Campinas</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Belo Horizonte</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>8450</v>
-      </c>
-      <c r="H3" t="n">
-        <v>760.4</v>
-      </c>
-      <c r="I3" t="n">
-        <v>320.5</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>aereo</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2026-02-05</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-02-06</t>
         </is>
       </c>
     </row>

</xml_diff>